<commit_message>
Fix a comment in the template.
</commit_message>
<xml_diff>
--- a/APmap-tmpl-v20250804.xlsx
+++ b/APmap-tmpl-v20250804.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\git\apmapdb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D7ED8B-4ECE-4D37-98D0-A9E72B6F7DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A762EC7C-59E4-40CA-BBB3-AC9ECE9A3B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6165" yWindow="3345" windowWidth="27015" windowHeight="19935" activeTab="1" xr2:uid="{1C09F2BD-4AD8-448C-9B67-4E49C39AE540}"/>
+    <workbookView xWindow="2450" yWindow="5510" windowWidth="21070" windowHeight="15370" activeTab="1" xr2:uid="{1C09F2BD-4AD8-448C-9B67-4E49C39AE540}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -734,7 +734,7 @@
     <t>CSV形式で提出する場合は、UTF-8エンコード、カンマ区切りにしてください。version行と、visibilityで始まるラベル行を、必ず含めてください。</t>
   </si>
   <si>
-    <t>versionの値は変更しないでください。</t>
+    <t>&lt; versionの値は変更しないでください。</t>
   </si>
 </sst>
 </file>
@@ -747,7 +747,7 @@
     <numFmt numFmtId="166" formatCode="0.0000000_ "/>
     <numFmt numFmtId="167" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -883,6 +883,13 @@
       <family val="2"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="0" tint="-0.14999847407452621"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -948,7 +955,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1123,6 +1130,9 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1442,11 +1452,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{564A7BE4-334C-448D-AEA0-3E36988B8C28}">
   <dimension ref="A2:I24"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="5"/>
-    <col min="2" max="2" width="90.28515625" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="9.1796875" style="5"/>
+    <col min="2" max="2" width="90.26953125" style="5" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="5"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9" ht="30">
@@ -1470,7 +1480,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="33">
+    <row r="10" spans="1:9" ht="32.5">
       <c r="B10" s="12" t="s">
         <v>21</v>
       </c>
@@ -1480,7 +1490,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="24">
+    <row r="15" spans="1:9" ht="24.5">
       <c r="A15" s="6"/>
       <c r="B15" s="6" t="s">
         <v>25</v>
@@ -1493,7 +1503,7 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9" ht="24">
+    <row r="16" spans="1:9" ht="24.5">
       <c r="A16" s="6"/>
       <c r="B16" s="6" t="s">
         <v>26</v>
@@ -1506,7 +1516,7 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" ht="24">
+    <row r="17" spans="1:9" ht="24.5">
       <c r="A17" s="6"/>
       <c r="B17" s="6" t="s">
         <v>11</v>
@@ -1519,7 +1529,7 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" spans="1:9" ht="24">
+    <row r="18" spans="1:9" ht="24.5">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1530,7 +1540,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" ht="24">
+    <row r="19" spans="1:9" ht="24.5">
       <c r="A19" s="6"/>
       <c r="B19" s="6" t="s">
         <v>90</v>
@@ -1543,7 +1553,7 @@
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
     </row>
-    <row r="20" spans="1:9" ht="24">
+    <row r="20" spans="1:9" ht="24.5">
       <c r="A20" s="6"/>
       <c r="B20" s="6" t="s">
         <v>27</v>
@@ -1556,7 +1566,7 @@
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
     </row>
-    <row r="21" spans="1:9" ht="24">
+    <row r="21" spans="1:9" ht="24.5">
       <c r="A21" s="6"/>
       <c r="B21" s="6" t="s">
         <v>10</v>
@@ -1569,7 +1579,7 @@
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
     </row>
-    <row r="22" spans="1:9" ht="24">
+    <row r="22" spans="1:9" ht="24.5">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1580,7 +1590,7 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" spans="1:9" ht="24">
+    <row r="23" spans="1:9" ht="24.5">
       <c r="A23" s="6"/>
       <c r="B23" s="6" t="s">
         <v>28</v>
@@ -1593,7 +1603,7 @@
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>
     </row>
-    <row r="24" spans="1:9" ht="24">
+    <row r="24" spans="1:9" ht="24.5">
       <c r="A24" s="6"/>
       <c r="B24" s="6" t="s">
         <v>9</v>
@@ -1618,44 +1628,46 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B35A389-7A8B-43CA-A10C-398A3B5E2FAA}">
-  <dimension ref="A1:Y22"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:Y21"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="13" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" style="13" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.26953125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.54296875" style="19" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="13.28515625" style="20" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="31" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" style="31" customWidth="1"/>
-    <col min="15" max="15" width="13.140625" style="31" customWidth="1"/>
-    <col min="16" max="16" width="34.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.140625" style="31" customWidth="1"/>
-    <col min="18" max="18" width="23.85546875" style="31" customWidth="1"/>
+    <col min="11" max="12" width="13.26953125" style="20" customWidth="1"/>
+    <col min="13" max="13" width="11.26953125" style="31" customWidth="1"/>
+    <col min="14" max="14" width="14.7265625" style="31" customWidth="1"/>
+    <col min="15" max="15" width="13.1796875" style="31" customWidth="1"/>
+    <col min="16" max="16" width="34.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.1796875" style="31" customWidth="1"/>
+    <col min="18" max="18" width="23.81640625" style="31" customWidth="1"/>
     <col min="19" max="19" width="15" style="31" customWidth="1"/>
-    <col min="20" max="20" width="58.28515625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="27.140625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.42578125" style="17" customWidth="1"/>
-    <col min="23" max="23" width="17.85546875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="25.28515625" style="47" customWidth="1"/>
-    <col min="25" max="25" width="11.7109375" style="1" customWidth="1"/>
-    <col min="26" max="16384" width="9.140625" style="1"/>
+    <col min="20" max="20" width="58.26953125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="27.1796875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="11.453125" style="17" customWidth="1"/>
+    <col min="23" max="23" width="17.81640625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="25.26953125" style="47" customWidth="1"/>
+    <col min="25" max="25" width="11.7265625" style="1" customWidth="1"/>
+    <col min="26" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="58" t="s">
         <v>99</v>
       </c>
-      <c r="C1" s="10"/>
+      <c r="C1" s="1" t="s">
+        <v>105</v>
+      </c>
       <c r="D1" s="2"/>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
@@ -1912,7 +1924,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="4" customFormat="1" ht="49.5">
+    <row r="6" spans="1:25" s="4" customFormat="1" ht="32">
       <c r="A6" s="27" t="s">
         <v>54</v>
       </c>
@@ -2204,11 +2216,6 @@
     <row r="21" spans="1:2">
       <c r="B21" s="1" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="B22" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>